<commit_message>
feat(qa): enhance Excel reports with domain-specific Reason for Passing and Validation Details columns
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Failed_Test_Cases.xlsx
+++ b/automation/reports/Excel/Failed_Test_Cases.xlsx
@@ -41,8 +41,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +75,7 @@
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -442,16 +442,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,17 +478,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Failure Reason</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Behavior</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Execution Time (s)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Failure Reason</t>
         </is>
       </c>
     </row>

</xml_diff>